<commit_message>
V6 Alpha1 implem suporte circular
</commit_message>
<xml_diff>
--- a/importacaoV5.xlsx
+++ b/importacaoV5.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="85">
   <si>
     <t>CAMPO</t>
   </si>
@@ -265,17 +265,29 @@
     <t>i</t>
   </si>
   <si>
-    <t>07A</t>
-  </si>
-  <si>
-    <t>07X</t>
+    <t>06X</t>
+  </si>
+  <si>
+    <t>LINHA_CIRCULAR</t>
+  </si>
+  <si>
+    <t>texto</t>
+  </si>
+  <si>
+    <t>true | false</t>
+  </si>
+  <si>
+    <t>hora | inteiro</t>
+  </si>
+  <si>
+    <t>true</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +333,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -450,7 +469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -555,6 +574,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1354,7 +1376,9 @@
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
+      <c r="E2" s="46" t="s">
+        <v>81</v>
+      </c>
       <c r="F2" s="43" t="s">
         <v>67</v>
       </c>
@@ -1528,7 +1552,9 @@
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="E3" s="46" t="s">
+        <v>81</v>
+      </c>
       <c r="F3" s="43">
         <v>410</v>
       </c>
@@ -1584,7 +1610,9 @@
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
+      <c r="E4" s="46" t="s">
+        <v>81</v>
+      </c>
       <c r="F4" s="43">
         <v>20</v>
       </c>
@@ -1674,7 +1702,9 @@
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
+      <c r="E5" s="46" t="s">
+        <v>81</v>
+      </c>
       <c r="F5" s="43">
         <v>61</v>
       </c>
@@ -1768,7 +1798,9 @@
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
+      <c r="E6" s="46" t="s">
+        <v>83</v>
+      </c>
       <c r="F6" s="43">
         <v>5</v>
       </c>
@@ -1862,7 +1894,9 @@
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
+      <c r="E7" s="46" t="s">
+        <v>83</v>
+      </c>
       <c r="F7" s="44">
         <v>1.5277777777777777E-2</v>
       </c>
@@ -1944,7 +1978,9 @@
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
+      <c r="E8" s="46" t="s">
+        <v>83</v>
+      </c>
       <c r="F8" s="44">
         <v>1.5277777777777777E-2</v>
       </c>
@@ -2034,7 +2070,9 @@
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
+      <c r="E9" s="46" t="s">
+        <v>81</v>
+      </c>
       <c r="F9" s="43">
         <v>51</v>
       </c>
@@ -2118,12 +2156,18 @@
       <c r="AV9" s="18"/>
     </row>
     <row r="10" spans="1:48" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
+      <c r="A10" s="13" t="s">
+        <v>80</v>
+      </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="43"/>
+      <c r="E10" s="46" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="43" t="s">
+        <v>84</v>
+      </c>
       <c r="G10" s="40"/>
       <c r="H10" s="20"/>
       <c r="I10" s="19">
@@ -2204,7 +2248,7 @@
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
+      <c r="E11" s="46"/>
       <c r="F11" s="43"/>
       <c r="G11" s="40"/>
       <c r="H11" s="20"/>
@@ -3506,7 +3550,9 @@
       <c r="L35" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="M35" s="37"/>
+      <c r="M35" s="37" t="s">
+        <v>79</v>
+      </c>
       <c r="N35" s="37"/>
       <c r="O35" s="37"/>
       <c r="P35" s="37">
@@ -3581,12 +3627,8 @@
       </c>
       <c r="J37" s="37"/>
       <c r="K37" s="45"/>
-      <c r="L37" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="M37" s="37" t="s">
-        <v>80</v>
-      </c>
+      <c r="L37" s="36"/>
+      <c r="M37" s="37"/>
       <c r="N37" s="37"/>
       <c r="O37" s="37"/>
       <c r="P37" s="37"/>

</xml_diff>